<commit_message>
feat: add traffic rules, rebel drivers and collisions
- Law-abiding drivers keep to speed limits (50 km/h on avenues,
  30 km/h on streets) and give way at junctions and roundabouts
- Rebel drivers ignore the rules and can crash; crashed cars are
  towed away after 30 s
- Count collisions, red lights run and speeding in experiments
- Run experiments in parallel, one run per processor core
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/CityMap.xlsx
+++ b/Assets/StreamingAssets/CityMap.xlsx
@@ -3699,7 +3699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>A cell that cars can enter from more than one direction is a junction. Cars take turns there: whoever has waited longest goes first.</t>
+          <t>A cell that cars can enter from more than one direction is a junction. Who goes first is decided by the traffic lights or, without lights, by the right of way (below).</t>
         </is>
       </c>
     </row>
@@ -3881,34 +3881,70 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Connections</t>
+          <t>Speed limits</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Every street cell must be reachable from every other street cell. In Unity, 'Traffic Simulation &gt; Check City Map' lists anything that goes nowhere.</t>
+          <t>Avenues (two or more lanes side by side) are 50 km/h; streets with one lane are 30 km/h. The cells right around a roundabout island are the roundabout, and are 30 km/h too.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Right of way</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>One cell is 1.2 Unity units (5.4 m). Cell A1 sits at the scene origin; columns go east (+X) and rows go south (-Z).</t>
+          <t>Where no traffic light decides: cars already in the roundabout go first, then cars going straight along the street (the arrow of the junction cell), then cars turning in. Between equals, whoever waited longest.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
+          <t>Rebels</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Law-abiding drivers (every taxi, most cars) follow all these rules and never crash. Rebel drivers ignore them and can crash; a crash blocks the street for 30 s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Connections</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Every street cell must be reachable from every other street cell. In Unity, 'Traffic Simulation &gt; Check City Map' lists anything that goes nowhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>One cell is 1.2 Unity units (5.4 m). Cell A1 sits at the scene origin; columns go east (+X) and rows go south (-Z).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
           <t>Where</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>The simulation reads the sheet named 'Map' of Assets/StreamingAssets/CityMap.xlsx when you press Play.</t>
         </is>

</xml_diff>